<commit_message>
chore(data): refresh FY2026 budget reference files and fixtures
- Replace versioned budget files (v3) with final FY2026 source files:
  01_EFIR_Revenue_FY2026.xlsx, 02_EFIR_Staff_Costs_FY2026.xlsx,
  03_EFIR_OpEx_FY2026.xlsx, 05_EFIR_Consolidated_Budget_FY2026v2.xlsx
- Remove superseded files: 01_v3, 02_DHG_v1, EFIR_Staff_Costs_Budget_V3
- Add DHG staffing.xlsx and staffing 2026-2027.xlsx source sheets
- Add School staff force master data files (FINAL QA + FINAL)
- Add Subjects directory: EFIR-Subjects-Coverage.xlsx + curriculum markdown
- Regenerate fy2026-dhg-structure.json and fy2026-staff-costs.json fixtures

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/budgets/EFIR_Consolidated_Monthly_Budget_FY2026.xlsx
+++ b/data/budgets/EFIR_Consolidated_Monthly_Budget_FY2026.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fakerhelali/Documents/EFIR Budget/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fakerhelali/Desktop/Budget 2026 EFIR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1728D8DF-883B-7747-9C78-765EFA69B3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C0DFA53-E071-1248-A49B-11DC74036D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IFRS Mapping" sheetId="1" r:id="rId1"/>
     <sheet name="IFRS Income Statement" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -786,14 +786,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1130,42 +1130,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1218,23 +1218,23 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -2127,23 +2127,23 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
@@ -2252,23 +2252,23 @@
       </c>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="22"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="O29" s="27"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
@@ -3137,23 +3137,23 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B48" s="22"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
-      <c r="N48" s="22"/>
-      <c r="O48" s="22"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
+      <c r="N48" s="27"/>
+      <c r="O48" s="27"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
@@ -4777,23 +4777,23 @@
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A83" s="21" t="s">
+      <c r="A83" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="B83" s="22"/>
-      <c r="C83" s="22"/>
-      <c r="D83" s="22"/>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="22"/>
-      <c r="H83" s="22"/>
-      <c r="I83" s="22"/>
-      <c r="J83" s="22"/>
-      <c r="K83" s="22"/>
-      <c r="L83" s="22"/>
-      <c r="M83" s="22"/>
-      <c r="N83" s="22"/>
-      <c r="O83" s="22"/>
+      <c r="B83" s="27"/>
+      <c r="C83" s="27"/>
+      <c r="D83" s="27"/>
+      <c r="E83" s="27"/>
+      <c r="F83" s="27"/>
+      <c r="G83" s="27"/>
+      <c r="H83" s="27"/>
+      <c r="I83" s="27"/>
+      <c r="J83" s="27"/>
+      <c r="K83" s="27"/>
+      <c r="L83" s="27"/>
+      <c r="M83" s="27"/>
+      <c r="N83" s="27"/>
+      <c r="O83" s="27"/>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
@@ -4908,23 +4908,23 @@
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A87" s="21" t="s">
+      <c r="A87" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="B87" s="22"/>
-      <c r="C87" s="22"/>
-      <c r="D87" s="22"/>
-      <c r="E87" s="22"/>
-      <c r="F87" s="22"/>
-      <c r="G87" s="22"/>
-      <c r="H87" s="22"/>
-      <c r="I87" s="22"/>
-      <c r="J87" s="22"/>
-      <c r="K87" s="22"/>
-      <c r="L87" s="22"/>
-      <c r="M87" s="22"/>
-      <c r="N87" s="22"/>
-      <c r="O87" s="22"/>
+      <c r="B87" s="27"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="27"/>
+      <c r="E87" s="27"/>
+      <c r="F87" s="27"/>
+      <c r="G87" s="27"/>
+      <c r="H87" s="27"/>
+      <c r="I87" s="27"/>
+      <c r="J87" s="27"/>
+      <c r="K87" s="27"/>
+      <c r="L87" s="27"/>
+      <c r="M87" s="27"/>
+      <c r="N87" s="27"/>
+      <c r="O87" s="27"/>
     </row>
     <row r="88" spans="1:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
@@ -5039,23 +5039,23 @@
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A91" s="21" t="s">
+      <c r="A91" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="B91" s="22"/>
-      <c r="C91" s="22"/>
-      <c r="D91" s="22"/>
-      <c r="E91" s="22"/>
-      <c r="F91" s="22"/>
-      <c r="G91" s="22"/>
-      <c r="H91" s="22"/>
-      <c r="I91" s="22"/>
-      <c r="J91" s="22"/>
-      <c r="K91" s="22"/>
-      <c r="L91" s="22"/>
-      <c r="M91" s="22"/>
-      <c r="N91" s="22"/>
-      <c r="O91" s="22"/>
+      <c r="B91" s="27"/>
+      <c r="C91" s="27"/>
+      <c r="D91" s="27"/>
+      <c r="E91" s="27"/>
+      <c r="F91" s="27"/>
+      <c r="G91" s="27"/>
+      <c r="H91" s="27"/>
+      <c r="I91" s="27"/>
+      <c r="J91" s="27"/>
+      <c r="K91" s="27"/>
+      <c r="L91" s="27"/>
+      <c r="M91" s="27"/>
+      <c r="N91" s="27"/>
+      <c r="O91" s="27"/>
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
@@ -5218,23 +5218,23 @@
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A96" s="21" t="s">
+      <c r="A96" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="B96" s="22"/>
-      <c r="C96" s="22"/>
-      <c r="D96" s="22"/>
-      <c r="E96" s="22"/>
-      <c r="F96" s="22"/>
-      <c r="G96" s="22"/>
-      <c r="H96" s="22"/>
-      <c r="I96" s="22"/>
-      <c r="J96" s="22"/>
-      <c r="K96" s="22"/>
-      <c r="L96" s="22"/>
-      <c r="M96" s="22"/>
-      <c r="N96" s="22"/>
-      <c r="O96" s="22"/>
+      <c r="B96" s="27"/>
+      <c r="C96" s="27"/>
+      <c r="D96" s="27"/>
+      <c r="E96" s="27"/>
+      <c r="F96" s="27"/>
+      <c r="G96" s="27"/>
+      <c r="H96" s="27"/>
+      <c r="I96" s="27"/>
+      <c r="J96" s="27"/>
+      <c r="K96" s="27"/>
+      <c r="L96" s="27"/>
+      <c r="M96" s="27"/>
+      <c r="N96" s="27"/>
+      <c r="O96" s="27"/>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
@@ -5530,40 +5530,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
@@ -5607,12 +5607,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>133</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>58209065.300000004</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>134</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v>8568791</v>
       </c>
     </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>135</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>1312800</v>
       </c>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>136</v>
       </c>
@@ -5840,7 +5840,7 @@
         <v>364479</v>
       </c>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>137</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>68455135.299999997</v>
       </c>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>138</v>
       </c>
@@ -6072,7 +6072,7 @@
         <f>SUM(B15:M15)</f>
         <v>-36892852.040000007</v>
       </c>
-      <c r="O15" s="28">
+      <c r="O15" s="21">
         <f>N15/$N$12</f>
         <v>-0.53853173872090887</v>
       </c>
@@ -6133,7 +6133,7 @@
         <f>SUM(B16:M16)</f>
         <v>-23590514.760000002</v>
       </c>
-      <c r="O16" s="28">
+      <c r="O16" s="21">
         <f t="shared" ref="O16:O17" si="3">N16/$N$12</f>
         <v>-0.34435507770583468</v>
       </c>
@@ -6194,12 +6194,12 @@
         <f>SUM(B17:M17)</f>
         <v>-5277816</v>
       </c>
-      <c r="O17" s="28">
+      <c r="O17" s="21">
         <f t="shared" si="3"/>
         <v>-7.7041249726298791E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>144</v>
       </c>
@@ -6312,7 +6312,7 @@
         <f>SUM(B19:M19)</f>
         <v>-66906376.759999983</v>
       </c>
-      <c r="O19" s="28">
+      <c r="O19" s="21">
         <f>N19/$N$12</f>
         <v>-0.97664467276786315</v>
       </c>
@@ -6373,17 +6373,17 @@
         <f>SUM(B21:M21)</f>
         <v>1599988.5799999982</v>
       </c>
-      <c r="O21" s="28">
+      <c r="O21" s="21">
         <f>N21/$N$12</f>
         <v>2.3355327232136559E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>148</v>
       </c>
@@ -6440,7 +6440,7 @@
         <v>599135.03999999992</v>
       </c>
     </row>
-    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>149</v>
       </c>
@@ -6553,7 +6553,7 @@
         <f>SUM(B26:M26)</f>
         <v>-1144715.1600000004</v>
       </c>
-      <c r="O26" s="28">
+      <c r="O26" s="21">
         <f>N26/$N$12</f>
         <v>-1.6709617483262034E-2</v>
       </c>
@@ -6671,7 +6671,7 @@
         <f>SUM(B29:M29)</f>
         <v>-287692.11</v>
       </c>
-      <c r="O29" s="28">
+      <c r="O29" s="21">
         <f>N29/$N$12</f>
         <v>-4.1994945808637172E-3</v>
       </c>
@@ -6739,94 +6739,94 @@
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="24"/>
-      <c r="N34" s="24"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+      <c r="N34" s="23"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
-      <c r="J35" s="24"/>
-      <c r="K35" s="24"/>
-      <c r="L35" s="24"/>
-      <c r="M35" s="24"/>
-      <c r="N35" s="24"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A36" s="27" t="s">
+      <c r="A36" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="24"/>
-      <c r="J36" s="24"/>
-      <c r="K36" s="24"/>
-      <c r="L36" s="24"/>
-      <c r="M36" s="24"/>
-      <c r="N36" s="24"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="23"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A37" s="27" t="s">
+      <c r="A37" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="24"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="24"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
-      <c r="J38" s="24"/>
-      <c r="K38" s="24"/>
-      <c r="L38" s="24"/>
-      <c r="M38" s="24"/>
-      <c r="N38" s="24"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="23"/>
+      <c r="N38" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>